<commit_message>
Atualiza catálogo do Facebook com os 22 produtos fitness da Winnek
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LTB4dkEdJS31EKKtoyhB9d
</commit_message>
<xml_diff>
--- a/catalogo_facebook_winnek.xlsx
+++ b/catalogo_facebook_winnek.xlsx
@@ -654,7 +654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC11"/>
+  <dimension ref="A1:AC24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12" defaultRowHeight="14.4" outlineLevelRow="0"/>
   <sheetData>
     <row r="1">
@@ -954,17 +954,17 @@
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t>MLB4014665095</t>
+          <t>MLB4398461911</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>Bicicleta Ergométrica Horizontal Magnética Winnek Monitor Digital 8 Niveis de ajustes Sensor de pulsaçao Pedal com Cinta Ajustavel</t>
+          <t>Bicicleta Spinning Winnek Enduro Com Roda de Inércia de 20kg e Bluetooth</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>Bicicleta ergométrica horizontal da Winnek com resistência magnética e 8 níveis de ajuste. Tem monitor digital, sensor de pulsação e pedais com cinta ajustável. Ideal para treinar em casa com conforto e segurança.</t>
+          <t>Bicicleta de spinning Winnek Enduro com roda de inércia de 20 kg e conexão Bluetooth. Pedalada firme e estável para treinos intensos em casa.</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
@@ -979,17 +979,17 @@
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>1600.00 BRL</t>
+          <t>2852.00 BRL</t>
         </is>
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>https://www.mercadolivre.com.br/bicicleta-ergometrica-horizontal-magnetica-winnek-monitor-digital-8-niveis-de-ajustes-sensor-de-pulsacao-pedal-com-cinta-ajustavel/p/MLB47419842?pdp_filters=item_id%3AMLB4014665095</t>
+          <t>https://www.mercadolivre.com.br/bicicleta-spinning-winnek-enduro-com-roda-de-inercia-de-20kg-e-bluetooth/p/MLB63673020?pdp_filters=item_id%3AMLB4398461911</t>
         </is>
       </c>
       <c r="H3" s="0" t="inlineStr">
         <is>
-          <t>https://http2.mlstatic.com/D_NQ_NP_2X_861719-MLA99989646517_112025-F.jpg</t>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_926199-MLA104268345393_012026-F.jpg</t>
         </is>
       </c>
       <c r="I3" s="0" t="inlineStr">
@@ -1006,7 +1006,7 @@
       <c r="L3" s="0" t="n"/>
       <c r="M3" s="0" t="inlineStr">
         <is>
-          <t>1297.00 BRL</t>
+          <t>1533.00 BRL</t>
         </is>
       </c>
       <c r="N3" s="0" t="n"/>
@@ -1025,7 +1025,11 @@
       </c>
       <c r="T3" s="0" t="n"/>
       <c r="U3" s="0" t="n"/>
-      <c r="V3" s="0" t="n"/>
+      <c r="V3" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
+        </is>
+      </c>
       <c r="W3" s="0" t="n"/>
       <c r="X3" s="0" t="n"/>
       <c r="Y3" s="0" t="n"/>
@@ -1037,17 +1041,17 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t>MLB4398461911</t>
+          <t>MLB6304284352</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>Bicicleta Spinning Winnek Enduro Com Roda de Inércia de 20kg e Bluetooth</t>
+          <t>Bicicleta Ergométrica Spinning Winnek SYNC Magnética, com Roda de Inércia 13kg e Bluetooth para App Fitshow</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>Bicicleta de spinning Winnek Enduro com roda de inércia de 20 kg e conexão Bluetooth. Pedalada firme e estável para treinos intensos em casa.</t>
+          <t>Bicicleta ergométrica de spinning Winnek SYNC com resistência magnética, roda de inércia de 13 kg e Bluetooth para o app Fitshow. Acompanhe seus treinos pelo celular.</t>
         </is>
       </c>
       <c r="D4" s="0" t="inlineStr">
@@ -1062,17 +1066,17 @@
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t>2852.00 BRL</t>
+          <t>3724.00 BRL</t>
         </is>
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>https://www.mercadolivre.com.br/bicicleta-spinning-winnek-enduro-com-roda-de-inercia-de-20kg-e-bluetooth/p/MLB63673020?pdp_filters=item_id%3AMLB4398461911</t>
+          <t>https://www.mercadolivre.com.br/bicicleta-ergometrica-spinning-winnek-sync-magnetica-com-roda-de-inercia-13kg-e-bluetooth-para-app-fitshow/p/MLB65112472?pdp_filters=item_id%3AMLB6304284352</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
         <is>
-          <t>https://http2.mlstatic.com/D_NQ_NP_2X_926199-MLA104268345393_012026-F.jpg</t>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_654810-MLA107970929851_032026-F.jpg</t>
         </is>
       </c>
       <c r="I4" s="0" t="inlineStr">
@@ -1087,7 +1091,7 @@
       </c>
       <c r="M4" s="0" t="inlineStr">
         <is>
-          <t>1533.00 BRL</t>
+          <t>2023.00 BRL</t>
         </is>
       </c>
       <c r="P4" s="0" t="inlineStr">
@@ -1098,23 +1102,28 @@
       <c r="S4" s="0" t="inlineStr">
         <is>
           <t>adult</t>
+        </is>
+      </c>
+      <c r="V4" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t>MLB7524577924</t>
+          <t>MLB4014665095</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>Bicicleta Ergométrica Spinning Winnek Effort 13kg Magnética Amarelo</t>
+          <t>Bicicleta Ergométrica Horizontal Magnética Winnek com Monitor Digital, 8 Níveis de Ajuste, Sensor de Pulsação e Pedal com Cinta Ajustável</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t>Bicicleta ergométrica de spinning Winnek Effort com roda de inércia de 13 kg e resistência magnética. Treino eficiente para pedalar em casa.</t>
+          <t>Bicicleta ergométrica horizontal da Winnek com resistência magnética e 8 níveis de ajuste. Tem monitor digital, sensor de pulsação e pedais com cinta ajustável. Ideal para treinar em casa com conforto e segurança.</t>
         </is>
       </c>
       <c r="D5" s="0" t="inlineStr">
@@ -1129,17 +1138,17 @@
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
-          <t>2079.00 BRL</t>
+          <t>1600.00 BRL</t>
         </is>
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>https://www.mercadolivre.com.br/bicicleta-ergometrica-spinning-winnek-effort-13kg-magnetica/up/MLBU4974574880?pdp_filters=item_id%3AMLB7524577924</t>
+          <t>https://www.mercadolivre.com.br/bicicleta-ergometrica-horizontal-magnetica-winnek-monitor-digital-8-niveis-de-ajustes-sensor-de-pulsacao-pedal-com-cinta-ajustavel/p/MLB47419842?pdp_filters=item_id%3AMLB4014665095</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
-          <t>https://http2.mlstatic.com/D_NQ_NP_2X_863595-MLB116788666459_082026-F.jpg</t>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_861719-MLA99989646517_112025-F.jpg</t>
         </is>
       </c>
       <c r="I5" s="0" t="inlineStr">
@@ -1154,7 +1163,7 @@
       </c>
       <c r="M5" s="0" t="inlineStr">
         <is>
-          <t>1564.00 BRL</t>
+          <t>1297.00 BRL</t>
         </is>
       </c>
       <c r="P5" s="0" t="inlineStr">
@@ -1162,31 +1171,31 @@
           <t>unisex</t>
         </is>
       </c>
-      <c r="Q5" s="0" t="inlineStr">
-        <is>
-          <t>Amarelo</t>
-        </is>
-      </c>
       <c r="S5" s="0" t="inlineStr">
         <is>
           <t>adult</t>
+        </is>
+      </c>
+      <c r="V5" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t>MLB6304284352</t>
+          <t>MLB7176942010</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>Bicicleta Ergométrica Spinning Winnek SYNC Magnética, com Roda de Inércia 13kg e Bluetooth para App Fitshow</t>
+          <t>Bicicleta Ergométrica Horizontal Winnek Magnética com Bluetooth e 8 Níveis de Resistência</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>Bicicleta ergométrica de spinning Winnek SYNC com resistência magnética, roda de inércia de 13 kg e Bluetooth para o app Fitshow. Acompanhe seus treinos pelo celular.</t>
+          <t>Bicicleta ergométrica horizontal Winnek com resistência magnética, Bluetooth e 8 níveis de resistência. Treino confortável para fazer em casa.</t>
         </is>
       </c>
       <c r="D6" s="0" t="inlineStr">
@@ -1201,17 +1210,17 @@
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t>3724.00 BRL</t>
+          <t>2497.00 BRL</t>
         </is>
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>https://www.mercadolivre.com.br/bicicleta-ergometrica-spinning-winnek-sync-magnetica-com-roda-de-inercia-13kg-e-bluetooth-para-app-fitshow/p/MLB65112472?pdp_filters=item_id%3AMLB6304284352</t>
+          <t>https://www.mercadolivre.com.br/bicicleta-ergometrica-horizontal-winnek-magnetica-com-bluetooth-e-8-niveis-de-resistencia/p/MLB75493180?pdp_filters=item_id%3AMLB7176942010</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
         <is>
-          <t>https://http2.mlstatic.com/D_NQ_NP_2X_654810-MLA107970929851_032026-F.jpg</t>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_649022-MLA113401835488_072026-F.jpg</t>
         </is>
       </c>
       <c r="I6" s="0" t="inlineStr">
@@ -1226,7 +1235,7 @@
       </c>
       <c r="M6" s="0" t="inlineStr">
         <is>
-          <t>2023.00 BRL</t>
+          <t>1648.00 BRL</t>
         </is>
       </c>
       <c r="P6" s="0" t="inlineStr">
@@ -1237,23 +1246,28 @@
       <c r="S6" s="0" t="inlineStr">
         <is>
           <t>adult</t>
+        </is>
+      </c>
+      <c r="V6" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>MLB5457027116</t>
+          <t>MLB6630914644</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>Bicicleta Ergométrica Spinning 8kg Roda Inércia Mecânica Ajustável Monitor Suporte Celular Tablet - WINNEK GLIDE PRETO E VERDE</t>
+          <t>Elíptico Magnético 3,5kg Winnek WNNK2032 Preto</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>Bicicleta ergométrica de spinning Winnek Glide com roda de inércia de 8 kg e resistência mecânica ajustável. Vem com monitor e suporte para celular ou tablet.</t>
+          <t>Elíptico magnético Winnek WNNK2032 com roda de inércia de 3,5 kg. Exercício completo e de baixo impacto para fazer em casa.</t>
         </is>
       </c>
       <c r="D7" s="0" t="inlineStr">
@@ -1268,17 +1282,17 @@
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>1624.00 BRL</t>
+          <t>1911.00 BRL</t>
         </is>
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>https://www.mercadolivre.com.br/bicicleta-ergometrica-spinning-8kg-roda-inercia-mecanica-ajustavel-monitor-suporte-celular-tablet-winnek-glide-preto-e-verde/p/MLB50873283?pdp_filters=item_id%3AMLB5457027116</t>
+          <t>https://www.mercadolivre.com.br/eliptico-magnetico-35kg-winnek-wnnk2032-cor-preto-preto/p/MLB68031865?pdp_filters=item_id%3AMLB6630914644</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t>https://http2.mlstatic.com/D_NQ_NP_2X_715766-MLA99743215589_112025-F.jpg</t>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_672208-MLA110471887973_042026-F.jpg</t>
         </is>
       </c>
       <c r="I7" s="0" t="inlineStr">
@@ -1288,12 +1302,12 @@
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Cardio &gt; Cardio Machines &gt; Exercise Bikes</t>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Cardio &gt; Cardio Machines &gt; Elliptical Trainers</t>
         </is>
       </c>
       <c r="M7" s="0" t="inlineStr">
         <is>
-          <t>919.08 BRL</t>
+          <t>1490.00 BRL</t>
         </is>
       </c>
       <c r="P7" s="0" t="inlineStr">
@@ -1303,29 +1317,34 @@
       </c>
       <c r="Q7" s="0" t="inlineStr">
         <is>
-          <t>Preto e verde</t>
+          <t>Preto</t>
         </is>
       </c>
       <c r="S7" s="0" t="inlineStr">
         <is>
           <t>adult</t>
+        </is>
+      </c>
+      <c r="V7" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>MLB6630914644</t>
+          <t>MLB5457027116</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>Elíptico Magnético 3,5kg Winnek Wnnk2032 Preto</t>
+          <t>Bicicleta Ergométrica Spinning 8kg Roda de Inércia Mecânica Ajustável com Monitor e Suporte para Celular/Tablet - Winnek Glide Preto e Verde</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>Elíptico magnético Winnek WNNK2032 com roda de inércia de 3,5 kg. Exercício completo e de baixo impacto para fazer em casa.</t>
+          <t>Bicicleta ergométrica de spinning Winnek Glide com roda de inércia de 8 kg e resistência mecânica ajustável. Vem com monitor e suporte para celular ou tablet.</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
@@ -1340,17 +1359,17 @@
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>1911.00 BRL</t>
+          <t>1624.00 BRL</t>
         </is>
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t>https://www.mercadolivre.com.br/eliptico-magnetico-35kg-winnek-wnnk2032-cor-preto-preto/p/MLB68031865?pdp_filters=item_id%3AMLB6630914644</t>
+          <t>https://www.mercadolivre.com.br/bicicleta-ergometrica-spinning-8kg-roda-inercia-mecanica-ajustavel-monitor-suporte-celular-tablet-winnek-glide-preto-e-verde/p/MLB50873283?pdp_filters=item_id%3AMLB5457027116</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
-          <t>https://http2.mlstatic.com/D_NQ_NP_2X_672208-MLA110471887973_042026-F.jpg</t>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_715766-MLA99743215589_112025-F.jpg</t>
         </is>
       </c>
       <c r="I8" s="0" t="inlineStr">
@@ -1360,12 +1379,12 @@
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Cardio &gt; Cardio Machines &gt; Elliptical Trainers</t>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Cardio &gt; Cardio Machines &gt; Exercise Bikes</t>
         </is>
       </c>
       <c r="M8" s="0" t="inlineStr">
         <is>
-          <t>1490.00 BRL</t>
+          <t>919.08 BRL</t>
         </is>
       </c>
       <c r="P8" s="0" t="inlineStr">
@@ -1375,29 +1394,34 @@
       </c>
       <c r="Q8" s="0" t="inlineStr">
         <is>
-          <t>Preto</t>
+          <t>Preto e verde</t>
         </is>
       </c>
       <c r="S8" s="0" t="inlineStr">
         <is>
           <t>adult</t>
+        </is>
+      </c>
+      <c r="V8" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>MLB6630730282</t>
+          <t>MLB7372176812</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>Elíptico Magnético Winnek WNNK2029 com Assento Ajustável e 4 Níveis de Resistência</t>
+          <t>Esteira Elétrica Winnek Rush 2.0HP Dobrável para Residências</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>Elíptico magnético Winnek WNNK2029 com assento ajustável e 4 níveis de resistência. Treino de baixo impacto para fazer em casa.</t>
+          <t>Esteira elétrica Winnek Rush com motor de 2.0 HP e estrutura dobrável. Ideal para caminhar e correr em casa e guardar ocupando menos espaço.</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
@@ -1412,17 +1436,17 @@
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>1911.00 BRL</t>
+          <t>2749.00 BRL</t>
         </is>
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>https://www.mercadolivre.com.br/eliptico-magnetico-winnek-wnnk2029-com-assento-ajustavel-e-4-niveis-de-resistencia/p/MLB68030935?pdp_filters=item_id%3AMLB6630730282</t>
+          <t>https://www.mercadolivre.com.br/esteira-eletrica-winnek-rush-20hp-dobravel-para-residencias/p/MLB76225543?pdp_filters=item_id%3AMLB7372176812</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t>https://http2.mlstatic.com/D_NQ_NP_2X_834525-MLA110516510369_042026-F.jpg</t>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_872188-MLA116463610984_092026-F.jpg</t>
         </is>
       </c>
       <c r="I9" s="0" t="inlineStr">
@@ -1432,12 +1456,12 @@
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Cardio &gt; Cardio Machines &gt; Elliptical Trainers</t>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Cardio &gt; Cardio Machines &gt; Treadmills</t>
         </is>
       </c>
       <c r="M9" s="0" t="inlineStr">
         <is>
-          <t>1490.00 BRL</t>
+          <t>1816.00 BRL</t>
         </is>
       </c>
       <c r="P9" s="0" t="inlineStr">
@@ -1448,23 +1472,28 @@
       <c r="S9" s="0" t="inlineStr">
         <is>
           <t>adult</t>
+        </is>
+      </c>
+      <c r="V9" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>MLB7176942010</t>
+          <t>MLB4453850007</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>Bicicleta Ergométrica Horizontal WINNEK Magnética com Bluetooth e 8 Níveis de Resistência</t>
+          <t>Bicicleta Ergométrica Spinning com Roda de Inércia de 13kg Mecânica Preto e Roxo com Suporte para Celular/Tablet - Winnek Spin Force</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>Bicicleta ergométrica horizontal Winnek com resistência magnética, Bluetooth e 8 níveis de resistência. Treino confortável para fazer em casa.</t>
+          <t>Bicicleta ergométrica de spinning Winnek Spin Force com roda de inércia de 13 kg e resistência mecânica. Vem com suporte para celular ou tablet para treinar assistindo suas aulas.</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -1479,17 +1508,17 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>2497.00 BRL</t>
+          <t>1928.00 BRL</t>
         </is>
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>https://www.mercadolivre.com.br/bicicleta-ergometrica-horizontal-winnek-magnetica-com-bluetooth-e-8-niveis-de-resistencia/p/MLB75493180?pdp_filters=item_id%3AMLB7176942010</t>
+          <t>https://www.mercadolivre.com.br/bicicleta-ergometrica-spinning-com-roda-inercia-de-13kg-mecanica-cor-preto-roxa-mecanica-suporte-para-celular-tablet-winnek-spin-force/p/MLB65104776?pdp_filters=item_id%3AMLB4453850007</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
         <is>
-          <t>https://http2.mlstatic.com/D_NQ_NP_2X_649022-MLA113401835488_072026-F.jpg</t>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_886296-MLA106197698211_012026-F.jpg</t>
         </is>
       </c>
       <c r="I10" s="0" t="inlineStr">
@@ -1504,7 +1533,7 @@
       </c>
       <c r="M10" s="0" t="inlineStr">
         <is>
-          <t>1648.00 BRL</t>
+          <t>1160.00 BRL</t>
         </is>
       </c>
       <c r="P10" s="0" t="inlineStr">
@@ -1512,9 +1541,19 @@
           <t>unisex</t>
         </is>
       </c>
+      <c r="Q10" s="0" t="inlineStr">
+        <is>
+          <t>Preto e roxo</t>
+        </is>
+      </c>
       <c r="S10" s="0" t="inlineStr">
         <is>
           <t>adult</t>
+        </is>
+      </c>
+      <c r="V10" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
         </is>
       </c>
     </row>
@@ -1579,9 +1618,1090 @@
           <t>unisex</t>
         </is>
       </c>
+      <c r="R11" s="0" t="inlineStr">
+        <is>
+          <t>18 kg</t>
+        </is>
+      </c>
       <c r="S11" s="0" t="inlineStr">
         <is>
           <t>adult</t>
+        </is>
+      </c>
+      <c r="V11" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>MLB6659598440</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>Bicicleta Ergométrica Winnek Spin Force WNNK1708 13kg Preto e Roxo</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Bicicleta ergométrica Winnek Spin Force WNNK1708 com roda de inércia de 13 kg. Treino de spinning completo para fazer em casa.</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>in stock</t>
+        </is>
+      </c>
+      <c r="E12" s="0" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F12" s="0" t="inlineStr">
+        <is>
+          <t>1703.00 BRL</t>
+        </is>
+      </c>
+      <c r="G12" s="0" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/bicicleta-ergometrica-winnek-13kg-preto-wnnk1708-spin-force-cor-preto-e-roxo/p/MLB66116565?pdp_filters=item_id%3AMLB6659598440</t>
+        </is>
+      </c>
+      <c r="H12" s="0" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_836280-MLA107908948901_032026-F.jpg</t>
+        </is>
+      </c>
+      <c r="I12" s="0" t="inlineStr">
+        <is>
+          <t>Winnek</t>
+        </is>
+      </c>
+      <c r="J12" s="0" t="inlineStr">
+        <is>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Cardio &gt; Cardio Machines &gt; Exercise Bikes</t>
+        </is>
+      </c>
+      <c r="M12" s="0" t="inlineStr">
+        <is>
+          <t>1184.00 BRL</t>
+        </is>
+      </c>
+      <c r="P12" s="0" t="inlineStr">
+        <is>
+          <t>unisex</t>
+        </is>
+      </c>
+      <c r="Q12" s="0" t="inlineStr">
+        <is>
+          <t>Preto e roxo</t>
+        </is>
+      </c>
+      <c r="S12" s="0" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="V12" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>MLB6630730282</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>Elíptico Magnético Winnek WNNK2029 com Assento Ajustável e 4 Níveis de Resistência</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Elíptico magnético Winnek WNNK2029 com assento ajustável e 4 níveis de resistência. Treino de baixo impacto para fazer em casa.</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>in stock</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F13" s="0" t="inlineStr">
+        <is>
+          <t>1911.00 BRL</t>
+        </is>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/eliptico-magnetico-winnek-wnnk2029-com-assento-ajustavel-e-4-niveis-de-resistencia/p/MLB68030935?pdp_filters=item_id%3AMLB6630730282</t>
+        </is>
+      </c>
+      <c r="H13" s="0" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_834525-MLA110516510369_042026-F.jpg</t>
+        </is>
+      </c>
+      <c r="I13" s="0" t="inlineStr">
+        <is>
+          <t>Winnek</t>
+        </is>
+      </c>
+      <c r="J13" s="0" t="inlineStr">
+        <is>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Cardio &gt; Cardio Machines &gt; Elliptical Trainers</t>
+        </is>
+      </c>
+      <c r="M13" s="0" t="inlineStr">
+        <is>
+          <t>1490.00 BRL</t>
+        </is>
+      </c>
+      <c r="P13" s="0" t="inlineStr">
+        <is>
+          <t>unisex</t>
+        </is>
+      </c>
+      <c r="S13" s="0" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="V13" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>MLB5456923612</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>Bicicleta Spinning com Roda de Inércia de 13kg Winnek Fitness Preto e Verde</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Bicicleta de spinning Winnek com roda de inércia de 13 kg. Pedalada estável para treinos intensos em casa.</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>in stock</t>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F14" s="0" t="inlineStr">
+        <is>
+          <t>2210.00 BRL</t>
+        </is>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/bicicleta-spinning-com-roda-de-inercia-de-13kg-winnek-fitness-preto-verde/p/MLB50871746?pdp_filters=item_id%3AMLB5456923612</t>
+        </is>
+      </c>
+      <c r="H14" s="0" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_852695-MLA108820349079_032026-F.jpg</t>
+        </is>
+      </c>
+      <c r="I14" s="0" t="inlineStr">
+        <is>
+          <t>Winnek</t>
+        </is>
+      </c>
+      <c r="J14" s="0" t="inlineStr">
+        <is>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Cardio &gt; Cardio Machines &gt; Exercise Bikes</t>
+        </is>
+      </c>
+      <c r="M14" s="0" t="inlineStr">
+        <is>
+          <t>1105.00 BRL</t>
+        </is>
+      </c>
+      <c r="P14" s="0" t="inlineStr">
+        <is>
+          <t>unisex</t>
+        </is>
+      </c>
+      <c r="Q14" s="0" t="inlineStr">
+        <is>
+          <t>Preto e verde</t>
+        </is>
+      </c>
+      <c r="S14" s="0" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="V14" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>MLB7716333218</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>Kettlebell Profissional Winnek FlexBell 6kg Azul - Macio, Anti-Impacto e Protege o Piso</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Kettlebell Winnek FlexBell de 6 kg com revestimento macio e anti-impacto. Protege o piso e não machuca, ideal para treinar em casa.</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>in stock</t>
+        </is>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F15" s="0" t="inlineStr">
+        <is>
+          <t>160.00 BRL</t>
+        </is>
+      </c>
+      <c r="G15" s="0" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/kettlebell-profissional-winnek-azul-6kg-flexbell-macio-anti-impacto-protege-o-piso-nao-machuca/p/MLB79878865?pdp_filters=item_id%3AMLB7716333218</t>
+        </is>
+      </c>
+      <c r="H15" s="0" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_623075-MLA118463130975_092026-F.jpg</t>
+        </is>
+      </c>
+      <c r="I15" s="0" t="inlineStr">
+        <is>
+          <t>Winnek</t>
+        </is>
+      </c>
+      <c r="J15" s="0" t="inlineStr">
+        <is>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Weight Lifting &gt; Free Weights</t>
+        </is>
+      </c>
+      <c r="M15" s="0" t="inlineStr">
+        <is>
+          <t>129.98 BRL</t>
+        </is>
+      </c>
+      <c r="O15" s="0" t="inlineStr">
+        <is>
+          <t>WINNEK-FLEXBELL</t>
+        </is>
+      </c>
+      <c r="P15" s="0" t="inlineStr">
+        <is>
+          <t>unisex</t>
+        </is>
+      </c>
+      <c r="Q15" s="0" t="inlineStr">
+        <is>
+          <t>Azul</t>
+        </is>
+      </c>
+      <c r="R15" s="0" t="inlineStr">
+        <is>
+          <t>6 kg</t>
+        </is>
+      </c>
+      <c r="S15" s="0" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="V15" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>MLB5304796855</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>Kettlebell Profissional Winnek FlexBell 10kg Roxo - Macio, Anti-Impacto e Protege o Piso</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Kettlebell Winnek FlexBell de 10 kg com revestimento macio e anti-impacto. Protege o piso e não machuca, ideal para treinar em casa.</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>in stock</t>
+        </is>
+      </c>
+      <c r="E16" s="0" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F16" s="0" t="inlineStr">
+        <is>
+          <t>219.00 BRL</t>
+        </is>
+      </c>
+      <c r="G16" s="0" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/kettlebell-profissional-winnek-roxo-10kg-flexbell-macio-anti-impacto-protege-o-piso-nao-machuca/p/MLB79878869?pdp_filters=item_id%3AMLB5304796855</t>
+        </is>
+      </c>
+      <c r="H16" s="0" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_832347-MLA116896357490_092026-F.jpg</t>
+        </is>
+      </c>
+      <c r="I16" s="0" t="inlineStr">
+        <is>
+          <t>Winnek</t>
+        </is>
+      </c>
+      <c r="J16" s="0" t="inlineStr">
+        <is>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Weight Lifting &gt; Free Weights</t>
+        </is>
+      </c>
+      <c r="M16" s="0" t="inlineStr">
+        <is>
+          <t>179.98 BRL</t>
+        </is>
+      </c>
+      <c r="O16" s="0" t="inlineStr">
+        <is>
+          <t>WINNEK-FLEXBELL</t>
+        </is>
+      </c>
+      <c r="P16" s="0" t="inlineStr">
+        <is>
+          <t>unisex</t>
+        </is>
+      </c>
+      <c r="Q16" s="0" t="inlineStr">
+        <is>
+          <t>Roxo</t>
+        </is>
+      </c>
+      <c r="R16" s="0" t="inlineStr">
+        <is>
+          <t>10 kg</t>
+        </is>
+      </c>
+      <c r="S16" s="0" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="V16" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>MLB5304834619</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>Kettlebell Profissional Winnek FlexBell 10kg Verde - Macio, Anti-Impacto e Protege o Piso</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Kettlebell Winnek FlexBell de 10 kg com revestimento macio e anti-impacto. Protege o piso e não machuca, ideal para treinar em casa.</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>in stock</t>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F17" s="0" t="inlineStr">
+        <is>
+          <t>219.00 BRL</t>
+        </is>
+      </c>
+      <c r="G17" s="0" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/kettlebell-profissional-winnek-verde-10kg-flexbell-macio-anti-impacto-protege-o-piso-nao-machuca/p/MLB79878868?pdp_filters=item_id%3AMLB5304834619</t>
+        </is>
+      </c>
+      <c r="H17" s="0" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_755441-MLA118457328641_092026-F.jpg</t>
+        </is>
+      </c>
+      <c r="I17" s="0" t="inlineStr">
+        <is>
+          <t>Winnek</t>
+        </is>
+      </c>
+      <c r="J17" s="0" t="inlineStr">
+        <is>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Weight Lifting &gt; Free Weights</t>
+        </is>
+      </c>
+      <c r="M17" s="0" t="inlineStr">
+        <is>
+          <t>179.98 BRL</t>
+        </is>
+      </c>
+      <c r="O17" s="0" t="inlineStr">
+        <is>
+          <t>WINNEK-FLEXBELL</t>
+        </is>
+      </c>
+      <c r="P17" s="0" t="inlineStr">
+        <is>
+          <t>unisex</t>
+        </is>
+      </c>
+      <c r="Q17" s="0" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="R17" s="0" t="inlineStr">
+        <is>
+          <t>10 kg</t>
+        </is>
+      </c>
+      <c r="S17" s="0" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="V17" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>MLB5304677863</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>Kettlebell Profissional Winnek FlexBell 4kg Azul - Macio, Anti-Impacto e Protege o Piso</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Kettlebell Winnek FlexBell de 4 kg com revestimento macio e anti-impacto. Protege o piso e não machuca, ideal para treinar em casa.</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>in stock</t>
+        </is>
+      </c>
+      <c r="E18" s="0" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F18" s="0" t="inlineStr">
+        <is>
+          <t>99.99 BRL</t>
+        </is>
+      </c>
+      <c r="G18" s="0" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/kettlebell-profissional-winnek-azul-4kg-flexbell-macio-anti-impacto-protege-o-piso-nao-machuca/p/MLB79878867?pdp_filters=item_id%3AMLB5304677863</t>
+        </is>
+      </c>
+      <c r="H18" s="0" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_909004-MLA116901740102_092026-F.jpg</t>
+        </is>
+      </c>
+      <c r="I18" s="0" t="inlineStr">
+        <is>
+          <t>Winnek</t>
+        </is>
+      </c>
+      <c r="J18" s="0" t="inlineStr">
+        <is>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Weight Lifting &gt; Free Weights</t>
+        </is>
+      </c>
+      <c r="M18" s="0" t="inlineStr">
+        <is>
+          <t>78.98 BRL</t>
+        </is>
+      </c>
+      <c r="O18" s="0" t="inlineStr">
+        <is>
+          <t>WINNEK-FLEXBELL</t>
+        </is>
+      </c>
+      <c r="P18" s="0" t="inlineStr">
+        <is>
+          <t>unisex</t>
+        </is>
+      </c>
+      <c r="Q18" s="0" t="inlineStr">
+        <is>
+          <t>Azul</t>
+        </is>
+      </c>
+      <c r="R18" s="0" t="inlineStr">
+        <is>
+          <t>4 kg</t>
+        </is>
+      </c>
+      <c r="S18" s="0" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="V18" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>MLB5310073885</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>Pesos de Pulso e Tornozelo Winnek Core Preto 4 lbs - Kit Fitness para Pilates e Musculação, Resistente à Água e ao Suor</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Kit de pesos de pulso e tornozelo Winnek Core para pilates e musculação. Material resistente à água e ao suor.</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>in stock</t>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F19" s="0" t="inlineStr">
+        <is>
+          <t>257.97 BRL</t>
+        </is>
+      </c>
+      <c r="G19" s="0" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/pesos-de-pulso-e-tornozelo-winnek-core-preto-kit-fitness-pilates-musculacao-material-resistente-agua-e-suor-preto-4-lbs/p/MLB79877213?pdp_filters=item_id%3AMLB5310073885</t>
+        </is>
+      </c>
+      <c r="H19" s="0" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_661685-MLA118449180903_092026-F.jpg</t>
+        </is>
+      </c>
+      <c r="I19" s="0" t="inlineStr">
+        <is>
+          <t>Winnek</t>
+        </is>
+      </c>
+      <c r="J19" s="0" t="inlineStr">
+        <is>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Exercise Weights</t>
+        </is>
+      </c>
+      <c r="M19" s="0" t="inlineStr">
+        <is>
+          <t>217.97 BRL</t>
+        </is>
+      </c>
+      <c r="O19" s="0" t="inlineStr">
+        <is>
+          <t>WINNEK-CORE</t>
+        </is>
+      </c>
+      <c r="P19" s="0" t="inlineStr">
+        <is>
+          <t>unisex</t>
+        </is>
+      </c>
+      <c r="Q19" s="0" t="inlineStr">
+        <is>
+          <t>Preto</t>
+        </is>
+      </c>
+      <c r="R19" s="0" t="inlineStr">
+        <is>
+          <t>4 lbs</t>
+        </is>
+      </c>
+      <c r="S19" s="0" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="V19" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>MLB5310123063</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>Pesos de Pulso e Tornozelo Winnek Core Bege 1 lb - Kit Fitness para Pilates e Musculação, Resistente à Água e ao Suor</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Kit de pesos de pulso e tornozelo Winnek Core para pilates e musculação. Material resistente à água e ao suor.</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>in stock</t>
+        </is>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F20" s="0" t="inlineStr">
+        <is>
+          <t>124.16 BRL</t>
+        </is>
+      </c>
+      <c r="G20" s="0" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/pesos-de-pulso-e-tornozelo-winnek-core-bege-kit-fitness-pilates-musculacao-material-resistente-agua-e-suor-bege-1lbs/p/MLB79877217?pdp_filters=item_id%3AMLB5310123063</t>
+        </is>
+      </c>
+      <c r="H20" s="0" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_607631-MLA116901979806_092026-F.jpg</t>
+        </is>
+      </c>
+      <c r="I20" s="0" t="inlineStr">
+        <is>
+          <t>Winnek</t>
+        </is>
+      </c>
+      <c r="J20" s="0" t="inlineStr">
+        <is>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Exercise Weights</t>
+        </is>
+      </c>
+      <c r="M20" s="0" t="inlineStr">
+        <is>
+          <t>107.97 BRL</t>
+        </is>
+      </c>
+      <c r="O20" s="0" t="inlineStr">
+        <is>
+          <t>WINNEK-CORE</t>
+        </is>
+      </c>
+      <c r="P20" s="0" t="inlineStr">
+        <is>
+          <t>unisex</t>
+        </is>
+      </c>
+      <c r="Q20" s="0" t="inlineStr">
+        <is>
+          <t>Bege</t>
+        </is>
+      </c>
+      <c r="R20" s="0" t="inlineStr">
+        <is>
+          <t>1 lb</t>
+        </is>
+      </c>
+      <c r="S20" s="0" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="V20" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>MLB7717821026</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>Peso Winnek Fistw Cinza 2 lbs</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Peso Winnek Fistw de 2 lbs para treinos de pilates, funcional e musculação.</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>in stock</t>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F21" s="0" t="inlineStr">
+        <is>
+          <t>149.90 BRL</t>
+        </is>
+      </c>
+      <c r="G21" s="0" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/peso-winnek-fistw-cinza-2lbs/p/MLB79877215?pdp_filters=item_id%3AMLB7717821026</t>
+        </is>
+      </c>
+      <c r="H21" s="0" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_780440-MLA118444514339_092026-F.jpg</t>
+        </is>
+      </c>
+      <c r="I21" s="0" t="inlineStr">
+        <is>
+          <t>Winnek</t>
+        </is>
+      </c>
+      <c r="J21" s="0" t="inlineStr">
+        <is>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Exercise Weights</t>
+        </is>
+      </c>
+      <c r="M21" s="0" t="inlineStr">
+        <is>
+          <t>126.69 BRL</t>
+        </is>
+      </c>
+      <c r="O21" s="0" t="inlineStr">
+        <is>
+          <t>WINNEK-FISTW</t>
+        </is>
+      </c>
+      <c r="P21" s="0" t="inlineStr">
+        <is>
+          <t>unisex</t>
+        </is>
+      </c>
+      <c r="Q21" s="0" t="inlineStr">
+        <is>
+          <t>Cinza</t>
+        </is>
+      </c>
+      <c r="R21" s="0" t="inlineStr">
+        <is>
+          <t>2 lbs</t>
+        </is>
+      </c>
+      <c r="S21" s="0" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="V21" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>MLB7717856922</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>Peso Winnek Fistw Rosa 2 lbs</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Peso Winnek Fistw de 2 lbs para treinos de pilates, funcional e musculação.</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>in stock</t>
+        </is>
+      </c>
+      <c r="E22" s="0" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F22" s="0" t="inlineStr">
+        <is>
+          <t>127.97 BRL</t>
+        </is>
+      </c>
+      <c r="G22" s="0" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/peso-winnek-fistw-rosa-2lbs/p/MLB79877216?pdp_filters=item_id%3AMLB7717856922</t>
+        </is>
+      </c>
+      <c r="H22" s="0" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_644047-MLA118445134923_092026-F.jpg</t>
+        </is>
+      </c>
+      <c r="I22" s="0" t="inlineStr">
+        <is>
+          <t>Winnek</t>
+        </is>
+      </c>
+      <c r="J22" s="0" t="inlineStr">
+        <is>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Exercise Weights</t>
+        </is>
+      </c>
+      <c r="M22" s="0" t="inlineStr">
+        <is>
+          <t>107.97 BRL</t>
+        </is>
+      </c>
+      <c r="O22" s="0" t="inlineStr">
+        <is>
+          <t>WINNEK-FISTW</t>
+        </is>
+      </c>
+      <c r="P22" s="0" t="inlineStr">
+        <is>
+          <t>unisex</t>
+        </is>
+      </c>
+      <c r="Q22" s="0" t="inlineStr">
+        <is>
+          <t>Rosa</t>
+        </is>
+      </c>
+      <c r="R22" s="0" t="inlineStr">
+        <is>
+          <t>2 lbs</t>
+        </is>
+      </c>
+      <c r="S22" s="0" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="V22" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>MLB7379472124</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>Banco para Bike Spinning Winnek</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Banco de reposição para bicicleta de spinning.</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>in stock</t>
+        </is>
+      </c>
+      <c r="E23" s="0" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F23" s="0" t="inlineStr">
+        <is>
+          <t>49.99 BRL</t>
+        </is>
+      </c>
+      <c r="G23" s="0" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/banco-para-bike-spinning/p/MLB76395903?pdp_filters=item_id%3AMLB7379472124</t>
+        </is>
+      </c>
+      <c r="H23" s="0" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_989772-MLA114303697886_082026-F.jpg</t>
+        </is>
+      </c>
+      <c r="I23" s="0" t="inlineStr">
+        <is>
+          <t>Winnek</t>
+        </is>
+      </c>
+      <c r="J23" s="0" t="inlineStr">
+        <is>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Cardio &gt; Cardio Machine Accessories</t>
+        </is>
+      </c>
+      <c r="M23" s="0" t="inlineStr">
+        <is>
+          <t>47.49 BRL</t>
+        </is>
+      </c>
+      <c r="P23" s="0" t="inlineStr">
+        <is>
+          <t>unisex</t>
+        </is>
+      </c>
+      <c r="S23" s="0" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="V23" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>MLB7524577924</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>Bicicleta Ergométrica Spinning Winnek Effort 13kg Magnética Amarelo</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Bicicleta ergométrica de spinning Winnek Effort com roda de inércia de 13 kg e resistência magnética. Treino eficiente para pedalar em casa.</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>in stock</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F24" s="0" t="inlineStr">
+        <is>
+          <t>2079.00 BRL</t>
+        </is>
+      </c>
+      <c r="G24" s="0" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/bicicleta-ergometrica-spinning-winnek-effort-13kg-magnetica/up/MLBU4974574880?pdp_filters=item_id%3AMLB7524577924</t>
+        </is>
+      </c>
+      <c r="H24" s="0" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_863595-MLB116788666459_082026-F.jpg</t>
+        </is>
+      </c>
+      <c r="I24" s="0" t="inlineStr">
+        <is>
+          <t>Winnek</t>
+        </is>
+      </c>
+      <c r="J24" s="0" t="inlineStr">
+        <is>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Cardio &gt; Cardio Machines &gt; Exercise Bikes</t>
+        </is>
+      </c>
+      <c r="M24" s="0" t="inlineStr">
+        <is>
+          <t>1564.00 BRL</t>
+        </is>
+      </c>
+      <c r="P24" s="0" t="inlineStr">
+        <is>
+          <t>unisex</t>
+        </is>
+      </c>
+      <c r="Q24" s="0" t="inlineStr">
+        <is>
+          <t>Amarelo</t>
+        </is>
+      </c>
+      <c r="S24" s="0" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="V24" s="0" t="inlineStr">
+        <is>
+          <t>BR::Frete grátis:0.00 BRL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Completa catálogo fitness da Winnek (25 produtos) e remove frete fixo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LTB4dkEdJS31EKKtoyhB9d
</commit_message>
<xml_diff>
--- a/catalogo_facebook_winnek.xlsx
+++ b/catalogo_facebook_winnek.xlsx
@@ -654,7 +654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC24"/>
+  <dimension ref="A1:AC27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12" defaultRowHeight="14.4" outlineLevelRow="0"/>
   <sheetData>
     <row r="1">
@@ -1025,11 +1025,7 @@
       </c>
       <c r="T3" s="0" t="n"/>
       <c r="U3" s="0" t="n"/>
-      <c r="V3" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
-        </is>
-      </c>
+      <c r="V3" s="0" t="n"/>
       <c r="W3" s="0" t="n"/>
       <c r="X3" s="0" t="n"/>
       <c r="Y3" s="0" t="n"/>
@@ -1104,11 +1100,6 @@
           <t>adult</t>
         </is>
       </c>
-      <c r="V4" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
@@ -1176,11 +1167,6 @@
           <t>adult</t>
         </is>
       </c>
-      <c r="V5" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
@@ -1248,11 +1234,6 @@
           <t>adult</t>
         </is>
       </c>
-      <c r="V6" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
@@ -1325,11 +1306,6 @@
           <t>adult</t>
         </is>
       </c>
-      <c r="V7" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
@@ -1402,11 +1378,6 @@
           <t>adult</t>
         </is>
       </c>
-      <c r="V8" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
@@ -1474,11 +1445,6 @@
           <t>adult</t>
         </is>
       </c>
-      <c r="V9" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
@@ -1551,11 +1517,6 @@
           <t>adult</t>
         </is>
       </c>
-      <c r="V10" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
@@ -1628,11 +1589,6 @@
           <t>adult</t>
         </is>
       </c>
-      <c r="V11" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
@@ -1705,11 +1661,6 @@
           <t>adult</t>
         </is>
       </c>
-      <c r="V12" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
@@ -1777,11 +1728,6 @@
           <t>adult</t>
         </is>
       </c>
-      <c r="V13" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
@@ -1854,11 +1800,6 @@
           <t>adult</t>
         </is>
       </c>
-      <c r="V14" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
@@ -1941,11 +1882,6 @@
           <t>adult</t>
         </is>
       </c>
-      <c r="V15" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
@@ -2028,11 +1964,6 @@
           <t>adult</t>
         </is>
       </c>
-      <c r="V16" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -2115,11 +2046,6 @@
           <t>adult</t>
         </is>
       </c>
-      <c r="V17" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
@@ -2202,11 +2128,6 @@
           <t>adult</t>
         </is>
       </c>
-      <c r="V18" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
@@ -2256,7 +2177,7 @@
       </c>
       <c r="J19" s="0" t="inlineStr">
         <is>
-          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Exercise Weights</t>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Weight Lifting &gt; Free Weights</t>
         </is>
       </c>
       <c r="M19" s="0" t="inlineStr">
@@ -2287,11 +2208,6 @@
       <c r="S19" s="0" t="inlineStr">
         <is>
           <t>adult</t>
-        </is>
-      </c>
-      <c r="V19" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
         </is>
       </c>
     </row>
@@ -2343,7 +2259,7 @@
       </c>
       <c r="J20" s="0" t="inlineStr">
         <is>
-          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Exercise Weights</t>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Weight Lifting &gt; Free Weights</t>
         </is>
       </c>
       <c r="M20" s="0" t="inlineStr">
@@ -2374,11 +2290,6 @@
       <c r="S20" s="0" t="inlineStr">
         <is>
           <t>adult</t>
-        </is>
-      </c>
-      <c r="V20" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
         </is>
       </c>
     </row>
@@ -2430,7 +2341,7 @@
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
-          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Exercise Weights</t>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Weight Lifting &gt; Free Weights</t>
         </is>
       </c>
       <c r="M21" s="0" t="inlineStr">
@@ -2461,11 +2372,6 @@
       <c r="S21" s="0" t="inlineStr">
         <is>
           <t>adult</t>
-        </is>
-      </c>
-      <c r="V21" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
         </is>
       </c>
     </row>
@@ -2517,7 +2423,7 @@
       </c>
       <c r="J22" s="0" t="inlineStr">
         <is>
-          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Exercise Weights</t>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Weight Lifting &gt; Free Weights</t>
         </is>
       </c>
       <c r="M22" s="0" t="inlineStr">
@@ -2548,11 +2454,6 @@
       <c r="S22" s="0" t="inlineStr">
         <is>
           <t>adult</t>
-        </is>
-      </c>
-      <c r="V22" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
         </is>
       </c>
     </row>
@@ -2622,86 +2523,282 @@
           <t>adult</t>
         </is>
       </c>
-      <c r="V23" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
+          <t>MLB7734620122</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>Kettlebell Winnek 4kg Rosa - Anti-Impacto, Não Machuca</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Kettlebell Winnek de 4 kg com revestimento anti-impacto que não machuca. Ideal para treinos funcionais em casa.</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>in stock</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F24" s="0" t="inlineStr">
+        <is>
+          <t>99.99 BRL</t>
+        </is>
+      </c>
+      <c r="G24" s="0" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/kettlebell-winnek-rosa-4-kg-antiimpacto-nao-machuca/up/MLBU5368772354?pdp_filters=item_id%3AMLB7734620122</t>
+        </is>
+      </c>
+      <c r="H24" s="0" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_836444-MLB118561702243_102026-F.jpg</t>
+        </is>
+      </c>
+      <c r="I24" s="0" t="inlineStr">
+        <is>
+          <t>Winnek</t>
+        </is>
+      </c>
+      <c r="J24" s="0" t="inlineStr">
+        <is>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Weight Lifting &gt; Free Weights</t>
+        </is>
+      </c>
+      <c r="P24" s="0" t="inlineStr">
+        <is>
+          <t>unisex</t>
+        </is>
+      </c>
+      <c r="Q24" s="0" t="inlineStr">
+        <is>
+          <t>Rosa</t>
+        </is>
+      </c>
+      <c r="R24" s="0" t="inlineStr">
+        <is>
+          <t>4 kg</t>
+        </is>
+      </c>
+      <c r="S24" s="0" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>MLB4338858483</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>Corda de Pular Winnek para Exercício Funcional, Ginástica e Treinos</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Corda de pular Winnek para treinos funcionais, ginástica e aquecimento. Leve e prática para levar para qualquer lugar.</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>in stock</t>
+        </is>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F25" s="0" t="inlineStr">
+        <is>
+          <t>22.94 BRL</t>
+        </is>
+      </c>
+      <c r="G25" s="0" t="inlineStr">
+        <is>
+          <t>https://produto.mercadolivre.com.br/MLB-4338858483-corda-de-pular-exercicio-funcional-ginastica-treinos-winnek-_JM</t>
+        </is>
+      </c>
+      <c r="H25" s="0" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_617775-MLB100061479049_122025-F.jpg</t>
+        </is>
+      </c>
+      <c r="I25" s="0" t="inlineStr">
+        <is>
+          <t>Winnek</t>
+        </is>
+      </c>
+      <c r="J25" s="0" t="inlineStr">
+        <is>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Jump Ropes</t>
+        </is>
+      </c>
+      <c r="M25" s="0" t="inlineStr">
+        <is>
+          <t>20.64 BRL</t>
+        </is>
+      </c>
+      <c r="P25" s="0" t="inlineStr">
+        <is>
+          <t>unisex</t>
+        </is>
+      </c>
+      <c r="S25" s="0" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>MLB5990864440</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>Corda de Pular Winnek para Exercício Funcional, Academia e Treinos</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Corda de pular Winnek para treinos funcionais e de academia. Leve e prática para levar para qualquer lugar.</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>in stock</t>
+        </is>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F26" s="0" t="inlineStr">
+        <is>
+          <t>20.34 BRL</t>
+        </is>
+      </c>
+      <c r="G26" s="0" t="inlineStr">
+        <is>
+          <t>https://produto.mercadolivre.com.br/MLB-5990864440-corda-de-pular-exercicio-funcional-academia-treinos-winnek-_JM</t>
+        </is>
+      </c>
+      <c r="H26" s="0" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_NQ_NP_2X_845800-MLB100059862387_122025-F.jpg</t>
+        </is>
+      </c>
+      <c r="I26" s="0" t="inlineStr">
+        <is>
+          <t>Winnek</t>
+        </is>
+      </c>
+      <c r="J26" s="0" t="inlineStr">
+        <is>
+          <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Jump Ropes</t>
+        </is>
+      </c>
+      <c r="M26" s="0" t="inlineStr">
+        <is>
+          <t>19.11 BRL</t>
+        </is>
+      </c>
+      <c r="P26" s="0" t="inlineStr">
+        <is>
+          <t>unisex</t>
+        </is>
+      </c>
+      <c r="S26" s="0" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
           <t>MLB7524577924</t>
         </is>
       </c>
-      <c r="B24" s="0" t="inlineStr">
+      <c r="B27" s="0" t="inlineStr">
         <is>
           <t>Bicicleta Ergométrica Spinning Winnek Effort 13kg Magnética Amarelo</t>
         </is>
       </c>
-      <c r="C24" s="0" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr">
         <is>
           <t>Bicicleta ergométrica de spinning Winnek Effort com roda de inércia de 13 kg e resistência magnética. Treino eficiente para pedalar em casa.</t>
         </is>
       </c>
-      <c r="D24" s="0" t="inlineStr">
+      <c r="D27" s="0" t="inlineStr">
         <is>
           <t>in stock</t>
         </is>
       </c>
-      <c r="E24" s="0" t="inlineStr">
+      <c r="E27" s="0" t="inlineStr">
         <is>
           <t>new</t>
         </is>
       </c>
-      <c r="F24" s="0" t="inlineStr">
+      <c r="F27" s="0" t="inlineStr">
         <is>
           <t>2079.00 BRL</t>
         </is>
       </c>
-      <c r="G24" s="0" t="inlineStr">
+      <c r="G27" s="0" t="inlineStr">
         <is>
           <t>https://www.mercadolivre.com.br/bicicleta-ergometrica-spinning-winnek-effort-13kg-magnetica/up/MLBU4974574880?pdp_filters=item_id%3AMLB7524577924</t>
         </is>
       </c>
-      <c r="H24" s="0" t="inlineStr">
+      <c r="H27" s="0" t="inlineStr">
         <is>
           <t>https://http2.mlstatic.com/D_NQ_NP_2X_863595-MLB116788666459_082026-F.jpg</t>
         </is>
       </c>
-      <c r="I24" s="0" t="inlineStr">
+      <c r="I27" s="0" t="inlineStr">
         <is>
           <t>Winnek</t>
         </is>
       </c>
-      <c r="J24" s="0" t="inlineStr">
+      <c r="J27" s="0" t="inlineStr">
         <is>
           <t>Sporting Goods &gt; Exercise &amp; Fitness &gt; Cardio &gt; Cardio Machines &gt; Exercise Bikes</t>
         </is>
       </c>
-      <c r="M24" s="0" t="inlineStr">
+      <c r="M27" s="0" t="inlineStr">
         <is>
           <t>1564.00 BRL</t>
         </is>
       </c>
-      <c r="P24" s="0" t="inlineStr">
+      <c r="P27" s="0" t="inlineStr">
         <is>
           <t>unisex</t>
         </is>
       </c>
-      <c r="Q24" s="0" t="inlineStr">
+      <c r="Q27" s="0" t="inlineStr">
         <is>
           <t>Amarelo</t>
         </is>
       </c>
-      <c r="S24" s="0" t="inlineStr">
+      <c r="S27" s="0" t="inlineStr">
         <is>
           <t>adult</t>
-        </is>
-      </c>
-      <c r="V24" s="0" t="inlineStr">
-        <is>
-          <t>BR::Frete grátis:0.00 BRL</t>
         </is>
       </c>
     </row>

</xml_diff>